<commit_message>
feat(11T + CCC): 11 Titulares mide solo AS+Almacén+Kiosco; tile CCC empresa real vs objetivo
- 11T: nuevo _mask_superficie_11t (Ramo AUTOSERVICIO o Subramo con AUTOSERVICIO
  -incluye Autoservicio Tradicional- + Almacén/Despensa + Kiosco/Maxikiosco;
  excluye On Premise, Vinotecas, Away, Mayoristas, Cash&Carry, resto tradicional).
  Aplicado en once_titulares, once_titulares_zona, bloque cierre_mes y _cierre_once_titulares.
- CCC empresa: gerencia_ccc_empresa reescrito -> CCC mes vivo (ventas.csv) por 5 canales
  de objccc.xlsx (por Ramo) vs objetivo; card nueva en portal + kcard real/obj/%.
- Objetivos del mes: objetivo 11T.xlsx actualizado; nuevo input objccc.xlsx.
- Validado con test_client (endpoints 200, filtro efectivo, totales reconcilian).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_INPUTS/objetivo 11T.xlsx
+++ b/01_INPUTS/objetivo 11T.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Orbit\MATINAL_PENAFLOR\01_INPUTS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E45725C-8FB5-495A-AC08-EEB2EF95F341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{937C5C1D-A6CC-4168-BB91-9599E2F0BF5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{2756557E-6E43-4FBF-8971-227ACF024C24}"/>
   </bookViews>
@@ -447,7 +447,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="1">
-        <v>639</v>
+        <v>318</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.25">
@@ -455,7 +455,7 @@
         <v>1</v>
       </c>
       <c r="C4" s="1">
-        <v>137</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
@@ -463,7 +463,7 @@
         <v>2</v>
       </c>
       <c r="C5" s="1">
-        <v>384</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
@@ -471,7 +471,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="1">
-        <v>440</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
@@ -479,7 +479,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="1">
-        <v>60</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
@@ -487,7 +487,7 @@
         <v>5</v>
       </c>
       <c r="C8" s="1">
-        <v>467</v>
+        <v>254</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
@@ -495,7 +495,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="1">
-        <v>317</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
@@ -503,7 +503,7 @@
         <v>7</v>
       </c>
       <c r="C10" s="1">
-        <v>396</v>
+        <v>199</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
@@ -511,7 +511,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="1">
-        <v>190</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
@@ -519,7 +519,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="1">
-        <v>400</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
@@ -527,7 +527,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="1">
-        <v>122</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>